<commit_message>
Add RPO engine to software model and build the Adobe FY2025 case
Adds a revenue-recognition/RPO (remaining performance obligation) engine to the software/SaaS builder and a real, source-addressed Adobe FY2025 case built on it. Every input is sourced to Adobe's actual 10-K XBRL company facts (CIK 0000796343); where a proxy is used (ARR has no fixed XBRL tag), the case documents the proxy's direction and measured error explicitly (-4.76% on modelled vs disclosed FY2025 revenue) rather than hiding it.
</commit_message>
<xml_diff>
--- a/31_Software_SaaS/_template_SOFTWARE.xlsx
+++ b/31_Software_SaaS/_template_SOFTWARE.xlsx
@@ -14,11 +14,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ARR Rollforward" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operating Model" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Economics" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule of 40" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RefreshLog" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RPO &amp; Bookings" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Economics" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule of 40" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RefreshLog" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="FS_MODEL_ID">'Institutional Surface'!$C$4</definedName>
@@ -153,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -171,9 +172,10 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -751,7 +753,248 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C14"/>
+  <dimension ref="B2:H10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="28" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Growth versus Profitability Trade-off</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Revenue growth</t>
+        </is>
+      </c>
+      <c r="C5" s="12">
+        <f>'ARR Rollforward'!C14</f>
+        <v/>
+      </c>
+      <c r="D5" s="12">
+        <f>IFERROR('Operating Model'!D7/'Operating Model'!C7-1,0)</f>
+        <v/>
+      </c>
+      <c r="E5" s="12">
+        <f>IFERROR('Operating Model'!E7/'Operating Model'!D7-1,0)</f>
+        <v/>
+      </c>
+      <c r="F5" s="12">
+        <f>IFERROR('Operating Model'!F7/'Operating Model'!E7-1,0)</f>
+        <v/>
+      </c>
+      <c r="G5" s="12">
+        <f>IFERROR('Operating Model'!G7/'Operating Model'!F7-1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>FCF margin</t>
+        </is>
+      </c>
+      <c r="C6" s="12">
+        <f>'Operating Model'!C24</f>
+        <v/>
+      </c>
+      <c r="D6" s="12">
+        <f>'Operating Model'!D24</f>
+        <v/>
+      </c>
+      <c r="E6" s="12">
+        <f>'Operating Model'!E24</f>
+        <v/>
+      </c>
+      <c r="F6" s="12">
+        <f>'Operating Model'!F24</f>
+        <v/>
+      </c>
+      <c r="G6" s="12">
+        <f>'Operating Model'!G24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Rule of 40 (growth + FCF margin)</t>
+        </is>
+      </c>
+      <c r="C7" s="12">
+        <f>C5+C6</f>
+        <v/>
+      </c>
+      <c r="D7" s="12">
+        <f>D5+D6</f>
+        <v/>
+      </c>
+      <c r="E7" s="12">
+        <f>E5+E6</f>
+        <v/>
+      </c>
+      <c r="F7" s="12">
+        <f>F5+F6</f>
+        <v/>
+      </c>
+      <c r="G7" s="12">
+        <f>G5+G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Non-GAAP operating margin</t>
+        </is>
+      </c>
+      <c r="C8" s="12">
+        <f>'Operating Model'!C20</f>
+        <v/>
+      </c>
+      <c r="D8" s="12">
+        <f>'Operating Model'!D20</f>
+        <v/>
+      </c>
+      <c r="E8" s="12">
+        <f>'Operating Model'!E20</f>
+        <v/>
+      </c>
+      <c r="F8" s="12">
+        <f>'Operating Model'!F20</f>
+        <v/>
+      </c>
+      <c r="G8" s="12">
+        <f>'Operating Model'!G20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Rule of 40 (growth + operating margin)</t>
+        </is>
+      </c>
+      <c r="C9" s="12">
+        <f>C5+C8</f>
+        <v/>
+      </c>
+      <c r="D9" s="12">
+        <f>D5+D8</f>
+        <v/>
+      </c>
+      <c r="E9" s="12">
+        <f>E5+E8</f>
+        <v/>
+      </c>
+      <c r="F9" s="12">
+        <f>F5+F8</f>
+        <v/>
+      </c>
+      <c r="G9" s="12">
+        <f>G5+G8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C10">
+        <f>IF(C7&gt;=0.4,"PASS",IF(C7&gt;=0.3,"REVIEW","BELOW"))</f>
+        <v/>
+      </c>
+      <c r="D10">
+        <f>IF(D7&gt;=0.4,"PASS",IF(D7&gt;=0.3,"REVIEW","BELOW"))</f>
+        <v/>
+      </c>
+      <c r="E10">
+        <f>IF(E7&gt;=0.4,"PASS",IF(E7&gt;=0.3,"REVIEW","BELOW"))</f>
+        <v/>
+      </c>
+      <c r="F10">
+        <f>IF(F7&gt;=0.4,"PASS",IF(F7&gt;=0.3,"REVIEW","BELOW"))</f>
+        <v/>
+      </c>
+      <c r="G10">
+        <f>IF(G7&gt;=0.4,"PASS",IF(G7&gt;=0.3,"REVIEW","BELOW"))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:H2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C10:G10">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>C10="PASS"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>C10="FAIL"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2">
+      <formula>C10="REVIEW"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="1">
+      <formula>C10="BREACH"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -880,11 +1123,55 @@
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
+          <t>RPO roll-forward reconciles (ending = beginning + bookings - revenue)</t>
+        </is>
+      </c>
+      <c r="C14">
+        <f>IF(MAX(ABS('RPO &amp; Bookings'!C7:G7-('RPO &amp; Bookings'!C6:G6+'RPO &amp; Bookings'!C8:G8-'RPO &amp; Bookings'!C5:G5)))&lt;0.000001,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Current RPO does not exceed total RPO</t>
+        </is>
+      </c>
+      <c r="C15">
+        <f>IF(MIN('RPO &amp; Bookings'!C12:G12)&gt;=-0.000001,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Contract liability does not exceed total RPO (unbilled RPO non-negative)</t>
+        </is>
+      </c>
+      <c r="C16">
+        <f>IF(MIN('RPO &amp; Bookings'!C14:G14)&gt;=-0.000001,"PASS","REVIEW")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Implied gross bookings positive (no negative-bookings year)</t>
+        </is>
+      </c>
+      <c r="C17">
+        <f>IF(MIN('RPO &amp; Bookings'!C8:G8)&gt;0,"PASS","REVIEW")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
           <t>Overall</t>
         </is>
       </c>
-      <c r="C14">
-        <f>IF(COUNTIF(C5:C13,"FAIL")&gt;0,"FAIL",IF(COUNTIF(C5:C13,"REVIEW")&gt;0,"REVIEW","PASS"))</f>
+      <c r="C18">
+        <f>IF(COUNTIF(C5:C17,"FAIL")&gt;0,"FAIL",IF(COUNTIF(C5:C17,"REVIEW")&gt;0,"REVIEW","PASS"))</f>
         <v/>
       </c>
     </row>
@@ -892,7 +1179,7 @@
   <mergeCells count="1">
     <mergeCell ref="B2:C2"/>
   </mergeCells>
-  <conditionalFormatting sqref="C5:C14">
+  <conditionalFormatting sqref="C5:C18">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>C5="PASS"</formula>
     </cfRule>
@@ -910,13 +1197,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E8"/>
+  <dimension ref="B2:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -956,88 +1243,132 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="17" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>ARR and retention disclosures</t>
         </is>
       </c>
-      <c r="C5" s="17" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>[10-K / 10-Q / shareholder letter]</t>
         </is>
       </c>
-      <c r="D5" s="17" t="inlineStr">
+      <c r="D5" s="18" t="inlineStr">
         <is>
           <t>[period]</t>
         </is>
       </c>
-      <c r="E5" s="17" t="inlineStr">
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>Beginning/ending ARR, NRR, customer counts</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Revenue disaggregation</t>
         </is>
       </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>[10-K revenue note]</t>
         </is>
       </c>
-      <c r="D6" s="17" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>[period]</t>
         </is>
       </c>
-      <c r="E6" s="17" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>Subscription versus services split and gross margin by type</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Stock-based compensation</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>[10-K equity note]</t>
         </is>
       </c>
-      <c r="D7" s="17" t="inlineStr">
+      <c r="D7" s="18" t="inlineStr">
         <is>
           <t>[period]</t>
         </is>
       </c>
-      <c r="E7" s="17" t="inlineStr">
+      <c r="E7" s="18" t="inlineStr">
         <is>
           <t>SBC by expense line</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Remaining performance obligations</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>[10-K revenue note / XBRL RevenueRemainingPerformanceObligation]</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>[period]</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>Total RPO and the portion expected to be recognised within twelve months</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Contract liabilities</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>[10-K balance sheet / XBRL ContractWithCustomerLiability]</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>[period]</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>Deferred revenue, used to split billed from unbilled RPO</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>Industry cost of capital and multiples</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C10" s="18" t="inlineStr">
         <is>
           <t>https://pages.stern.nyu.edu/~adamodar/New_Home_Page/data.html</t>
         </is>
       </c>
-      <c r="D8" s="17" t="inlineStr">
+      <c r="D10" s="18" t="inlineStr">
         <is>
           <t>[annual]</t>
         </is>
       </c>
-      <c r="E8" s="17" t="inlineStr">
+      <c r="E10" s="18" t="inlineStr">
         <is>
           <t>Software industry margins, betas, and multiple ranges for driver grounding</t>
         </is>
@@ -1051,7 +1382,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1109,204 +1440,204 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="18" t="n"/>
-      <c r="C5" s="18" t="n"/>
-      <c r="D5" s="18" t="n"/>
-      <c r="E5" s="18" t="n"/>
-      <c r="F5" s="18" t="n"/>
-      <c r="G5" s="18" t="n"/>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="19" t="n"/>
+      <c r="D5" s="19" t="n"/>
+      <c r="E5" s="19" t="n"/>
+      <c r="F5" s="19" t="n"/>
+      <c r="G5" s="19" t="n"/>
     </row>
     <row r="6">
-      <c r="B6" s="18" t="n"/>
-      <c r="C6" s="18" t="n"/>
-      <c r="D6" s="18" t="n"/>
-      <c r="E6" s="18" t="n"/>
-      <c r="F6" s="18" t="n"/>
-      <c r="G6" s="18" t="n"/>
+      <c r="B6" s="19" t="n"/>
+      <c r="C6" s="19" t="n"/>
+      <c r="D6" s="19" t="n"/>
+      <c r="E6" s="19" t="n"/>
+      <c r="F6" s="19" t="n"/>
+      <c r="G6" s="19" t="n"/>
     </row>
     <row r="7">
-      <c r="B7" s="18" t="n"/>
-      <c r="C7" s="18" t="n"/>
-      <c r="D7" s="18" t="n"/>
-      <c r="E7" s="18" t="n"/>
-      <c r="F7" s="18" t="n"/>
-      <c r="G7" s="18" t="n"/>
+      <c r="B7" s="19" t="n"/>
+      <c r="C7" s="19" t="n"/>
+      <c r="D7" s="19" t="n"/>
+      <c r="E7" s="19" t="n"/>
+      <c r="F7" s="19" t="n"/>
+      <c r="G7" s="19" t="n"/>
     </row>
     <row r="8">
-      <c r="B8" s="18" t="n"/>
-      <c r="C8" s="18" t="n"/>
-      <c r="D8" s="18" t="n"/>
-      <c r="E8" s="18" t="n"/>
-      <c r="F8" s="18" t="n"/>
-      <c r="G8" s="18" t="n"/>
+      <c r="B8" s="19" t="n"/>
+      <c r="C8" s="19" t="n"/>
+      <c r="D8" s="19" t="n"/>
+      <c r="E8" s="19" t="n"/>
+      <c r="F8" s="19" t="n"/>
+      <c r="G8" s="19" t="n"/>
     </row>
     <row r="9">
-      <c r="B9" s="18" t="n"/>
-      <c r="C9" s="18" t="n"/>
-      <c r="D9" s="18" t="n"/>
-      <c r="E9" s="18" t="n"/>
-      <c r="F9" s="18" t="n"/>
-      <c r="G9" s="18" t="n"/>
+      <c r="B9" s="19" t="n"/>
+      <c r="C9" s="19" t="n"/>
+      <c r="D9" s="19" t="n"/>
+      <c r="E9" s="19" t="n"/>
+      <c r="F9" s="19" t="n"/>
+      <c r="G9" s="19" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" s="18" t="n"/>
-      <c r="C10" s="18" t="n"/>
-      <c r="D10" s="18" t="n"/>
-      <c r="E10" s="18" t="n"/>
-      <c r="F10" s="18" t="n"/>
-      <c r="G10" s="18" t="n"/>
+      <c r="B10" s="19" t="n"/>
+      <c r="C10" s="19" t="n"/>
+      <c r="D10" s="19" t="n"/>
+      <c r="E10" s="19" t="n"/>
+      <c r="F10" s="19" t="n"/>
+      <c r="G10" s="19" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="18" t="n"/>
-      <c r="C11" s="18" t="n"/>
-      <c r="D11" s="18" t="n"/>
-      <c r="E11" s="18" t="n"/>
-      <c r="F11" s="18" t="n"/>
-      <c r="G11" s="18" t="n"/>
+      <c r="B11" s="19" t="n"/>
+      <c r="C11" s="19" t="n"/>
+      <c r="D11" s="19" t="n"/>
+      <c r="E11" s="19" t="n"/>
+      <c r="F11" s="19" t="n"/>
+      <c r="G11" s="19" t="n"/>
     </row>
     <row r="12">
-      <c r="B12" s="18" t="n"/>
-      <c r="C12" s="18" t="n"/>
-      <c r="D12" s="18" t="n"/>
-      <c r="E12" s="18" t="n"/>
-      <c r="F12" s="18" t="n"/>
-      <c r="G12" s="18" t="n"/>
+      <c r="B12" s="19" t="n"/>
+      <c r="C12" s="19" t="n"/>
+      <c r="D12" s="19" t="n"/>
+      <c r="E12" s="19" t="n"/>
+      <c r="F12" s="19" t="n"/>
+      <c r="G12" s="19" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="18" t="n"/>
-      <c r="C13" s="18" t="n"/>
-      <c r="D13" s="18" t="n"/>
-      <c r="E13" s="18" t="n"/>
-      <c r="F13" s="18" t="n"/>
-      <c r="G13" s="18" t="n"/>
+      <c r="B13" s="19" t="n"/>
+      <c r="C13" s="19" t="n"/>
+      <c r="D13" s="19" t="n"/>
+      <c r="E13" s="19" t="n"/>
+      <c r="F13" s="19" t="n"/>
+      <c r="G13" s="19" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="18" t="n"/>
-      <c r="C14" s="18" t="n"/>
-      <c r="D14" s="18" t="n"/>
-      <c r="E14" s="18" t="n"/>
-      <c r="F14" s="18" t="n"/>
-      <c r="G14" s="18" t="n"/>
+      <c r="B14" s="19" t="n"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="19" t="n"/>
+      <c r="E14" s="19" t="n"/>
+      <c r="F14" s="19" t="n"/>
+      <c r="G14" s="19" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="18" t="n"/>
-      <c r="C15" s="18" t="n"/>
-      <c r="D15" s="18" t="n"/>
-      <c r="E15" s="18" t="n"/>
-      <c r="F15" s="18" t="n"/>
-      <c r="G15" s="18" t="n"/>
+      <c r="B15" s="19" t="n"/>
+      <c r="C15" s="19" t="n"/>
+      <c r="D15" s="19" t="n"/>
+      <c r="E15" s="19" t="n"/>
+      <c r="F15" s="19" t="n"/>
+      <c r="G15" s="19" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="18" t="n"/>
-      <c r="C16" s="18" t="n"/>
-      <c r="D16" s="18" t="n"/>
-      <c r="E16" s="18" t="n"/>
-      <c r="F16" s="18" t="n"/>
-      <c r="G16" s="18" t="n"/>
+      <c r="B16" s="19" t="n"/>
+      <c r="C16" s="19" t="n"/>
+      <c r="D16" s="19" t="n"/>
+      <c r="E16" s="19" t="n"/>
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="19" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="18" t="n"/>
-      <c r="C17" s="18" t="n"/>
-      <c r="D17" s="18" t="n"/>
-      <c r="E17" s="18" t="n"/>
-      <c r="F17" s="18" t="n"/>
-      <c r="G17" s="18" t="n"/>
+      <c r="B17" s="19" t="n"/>
+      <c r="C17" s="19" t="n"/>
+      <c r="D17" s="19" t="n"/>
+      <c r="E17" s="19" t="n"/>
+      <c r="F17" s="19" t="n"/>
+      <c r="G17" s="19" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="18" t="n"/>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="18" t="n"/>
-      <c r="E18" s="18" t="n"/>
-      <c r="F18" s="18" t="n"/>
-      <c r="G18" s="18" t="n"/>
+      <c r="B18" s="19" t="n"/>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="19" t="n"/>
+      <c r="E18" s="19" t="n"/>
+      <c r="F18" s="19" t="n"/>
+      <c r="G18" s="19" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="18" t="n"/>
-      <c r="C19" s="18" t="n"/>
-      <c r="D19" s="18" t="n"/>
-      <c r="E19" s="18" t="n"/>
-      <c r="F19" s="18" t="n"/>
-      <c r="G19" s="18" t="n"/>
+      <c r="B19" s="19" t="n"/>
+      <c r="C19" s="19" t="n"/>
+      <c r="D19" s="19" t="n"/>
+      <c r="E19" s="19" t="n"/>
+      <c r="F19" s="19" t="n"/>
+      <c r="G19" s="19" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="18" t="n"/>
-      <c r="C20" s="18" t="n"/>
-      <c r="D20" s="18" t="n"/>
-      <c r="E20" s="18" t="n"/>
-      <c r="F20" s="18" t="n"/>
-      <c r="G20" s="18" t="n"/>
+      <c r="B20" s="19" t="n"/>
+      <c r="C20" s="19" t="n"/>
+      <c r="D20" s="19" t="n"/>
+      <c r="E20" s="19" t="n"/>
+      <c r="F20" s="19" t="n"/>
+      <c r="G20" s="19" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="18" t="n"/>
-      <c r="C21" s="18" t="n"/>
-      <c r="D21" s="18" t="n"/>
-      <c r="E21" s="18" t="n"/>
-      <c r="F21" s="18" t="n"/>
-      <c r="G21" s="18" t="n"/>
+      <c r="B21" s="19" t="n"/>
+      <c r="C21" s="19" t="n"/>
+      <c r="D21" s="19" t="n"/>
+      <c r="E21" s="19" t="n"/>
+      <c r="F21" s="19" t="n"/>
+      <c r="G21" s="19" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="18" t="n"/>
-      <c r="C22" s="18" t="n"/>
-      <c r="D22" s="18" t="n"/>
-      <c r="E22" s="18" t="n"/>
-      <c r="F22" s="18" t="n"/>
-      <c r="G22" s="18" t="n"/>
+      <c r="B22" s="19" t="n"/>
+      <c r="C22" s="19" t="n"/>
+      <c r="D22" s="19" t="n"/>
+      <c r="E22" s="19" t="n"/>
+      <c r="F22" s="19" t="n"/>
+      <c r="G22" s="19" t="n"/>
     </row>
     <row r="23">
-      <c r="B23" s="18" t="n"/>
-      <c r="C23" s="18" t="n"/>
-      <c r="D23" s="18" t="n"/>
-      <c r="E23" s="18" t="n"/>
-      <c r="F23" s="18" t="n"/>
-      <c r="G23" s="18" t="n"/>
+      <c r="B23" s="19" t="n"/>
+      <c r="C23" s="19" t="n"/>
+      <c r="D23" s="19" t="n"/>
+      <c r="E23" s="19" t="n"/>
+      <c r="F23" s="19" t="n"/>
+      <c r="G23" s="19" t="n"/>
     </row>
     <row r="24">
-      <c r="B24" s="18" t="n"/>
-      <c r="C24" s="18" t="n"/>
-      <c r="D24" s="18" t="n"/>
-      <c r="E24" s="18" t="n"/>
-      <c r="F24" s="18" t="n"/>
-      <c r="G24" s="18" t="n"/>
+      <c r="B24" s="19" t="n"/>
+      <c r="C24" s="19" t="n"/>
+      <c r="D24" s="19" t="n"/>
+      <c r="E24" s="19" t="n"/>
+      <c r="F24" s="19" t="n"/>
+      <c r="G24" s="19" t="n"/>
     </row>
     <row r="25">
-      <c r="B25" s="18" t="n"/>
-      <c r="C25" s="18" t="n"/>
-      <c r="D25" s="18" t="n"/>
-      <c r="E25" s="18" t="n"/>
-      <c r="F25" s="18" t="n"/>
-      <c r="G25" s="18" t="n"/>
+      <c r="B25" s="19" t="n"/>
+      <c r="C25" s="19" t="n"/>
+      <c r="D25" s="19" t="n"/>
+      <c r="E25" s="19" t="n"/>
+      <c r="F25" s="19" t="n"/>
+      <c r="G25" s="19" t="n"/>
     </row>
     <row r="26">
-      <c r="B26" s="18" t="n"/>
-      <c r="C26" s="18" t="n"/>
-      <c r="D26" s="18" t="n"/>
-      <c r="E26" s="18" t="n"/>
-      <c r="F26" s="18" t="n"/>
-      <c r="G26" s="18" t="n"/>
+      <c r="B26" s="19" t="n"/>
+      <c r="C26" s="19" t="n"/>
+      <c r="D26" s="19" t="n"/>
+      <c r="E26" s="19" t="n"/>
+      <c r="F26" s="19" t="n"/>
+      <c r="G26" s="19" t="n"/>
     </row>
     <row r="27">
-      <c r="B27" s="18" t="n"/>
-      <c r="C27" s="18" t="n"/>
-      <c r="D27" s="18" t="n"/>
-      <c r="E27" s="18" t="n"/>
-      <c r="F27" s="18" t="n"/>
-      <c r="G27" s="18" t="n"/>
+      <c r="B27" s="19" t="n"/>
+      <c r="C27" s="19" t="n"/>
+      <c r="D27" s="19" t="n"/>
+      <c r="E27" s="19" t="n"/>
+      <c r="F27" s="19" t="n"/>
+      <c r="G27" s="19" t="n"/>
     </row>
     <row r="28">
-      <c r="B28" s="18" t="n"/>
-      <c r="C28" s="18" t="n"/>
-      <c r="D28" s="18" t="n"/>
-      <c r="E28" s="18" t="n"/>
-      <c r="F28" s="18" t="n"/>
-      <c r="G28" s="18" t="n"/>
+      <c r="B28" s="19" t="n"/>
+      <c r="C28" s="19" t="n"/>
+      <c r="D28" s="19" t="n"/>
+      <c r="E28" s="19" t="n"/>
+      <c r="F28" s="19" t="n"/>
+      <c r="G28" s="19" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="18" t="n"/>
-      <c r="C29" s="18" t="n"/>
-      <c r="D29" s="18" t="n"/>
-      <c r="E29" s="18" t="n"/>
-      <c r="F29" s="18" t="n"/>
-      <c r="G29" s="18" t="n"/>
+      <c r="B29" s="19" t="n"/>
+      <c r="C29" s="19" t="n"/>
+      <c r="D29" s="19" t="n"/>
+      <c r="E29" s="19" t="n"/>
+      <c r="F29" s="19" t="n"/>
+      <c r="G29" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1333,125 +1664,125 @@
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" s="19" t="inlineStr">
+      <c r="B2" s="20" t="inlineStr">
         <is>
           <t>Software &amp; SaaS — Institutional Decision Surface</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>Model ID</t>
         </is>
       </c>
-      <c r="C4" s="21" t="inlineStr">
+      <c r="C4" s="22" t="inlineStr">
         <is>
           <t>31</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>Domain</t>
         </is>
       </c>
-      <c r="C5" s="21" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>Software &amp; SaaS</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>Declared maturity</t>
         </is>
       </c>
-      <c r="C6" s="21" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>M1</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>Canonical builder</t>
         </is>
       </c>
-      <c r="C7" s="21" t="inlineStr">
+      <c r="C7" s="22" t="inlineStr">
         <is>
           <t>tools/builders/build_software_saas_institutional.py</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="20" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>Decision arena</t>
         </is>
       </c>
-      <c r="C8" s="21" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>management team, board, public-market investors and growth-equity investment committee</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>Committee artifact</t>
         </is>
       </c>
-      <c r="C9" s="21" t="inlineStr">
+      <c r="C9" s="22" t="inlineStr">
         <is>
           <t>quarterly ARR and retention review pack</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>Operating cadence</t>
         </is>
       </c>
-      <c r="C10" s="21" t="inlineStr">
+      <c r="C10" s="22" t="inlineStr">
         <is>
           <t>quarterly earnings and ARR reporting; annual plan and long-range model refresh</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="22" t="inlineStr">
+      <c r="B12" s="23" t="inlineStr">
         <is>
           <t>Key decision outputs</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="23" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C13" s="23" t="inlineStr">
+      <c r="C13" s="24" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="D13" s="23" t="inlineStr">
+      <c r="D13" s="24" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="E13" s="23" t="inlineStr">
+      <c r="E13" s="24" t="inlineStr">
         <is>
           <t>Evidence / location</t>
         </is>
       </c>
-      <c r="F13" s="23" t="inlineStr">
+      <c r="F13" s="24" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -1543,34 +1874,34 @@
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="22" t="inlineStr">
+      <c r="B20" s="23" t="inlineStr">
         <is>
           <t>Insider questions</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="23" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C21" s="23" t="inlineStr">
+      <c r="C21" s="24" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="D21" s="23" t="inlineStr">
+      <c r="D21" s="24" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="E21" s="23" t="inlineStr">
+      <c r="E21" s="24" t="inlineStr">
         <is>
           <t>Evidence / location</t>
         </is>
       </c>
-      <c r="F21" s="23" t="inlineStr">
+      <c r="F21" s="24" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -1662,34 +1993,34 @@
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="22" t="inlineStr">
+      <c r="B28" s="23" t="inlineStr">
         <is>
           <t>Scenario families</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="23" t="inlineStr">
+      <c r="B29" s="24" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C29" s="23" t="inlineStr">
+      <c r="C29" s="24" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="D29" s="23" t="inlineStr">
+      <c r="D29" s="24" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="E29" s="23" t="inlineStr">
+      <c r="E29" s="24" t="inlineStr">
         <is>
           <t>Evidence / location</t>
         </is>
       </c>
-      <c r="F29" s="23" t="inlineStr">
+      <c r="F29" s="24" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -1781,34 +2112,34 @@
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="22" t="inlineStr">
+      <c r="B36" s="23" t="inlineStr">
         <is>
           <t>Primary diligence documents</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="23" t="inlineStr">
+      <c r="B37" s="24" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C37" s="23" t="inlineStr">
+      <c r="C37" s="24" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="D37" s="23" t="inlineStr">
+      <c r="D37" s="24" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="E37" s="23" t="inlineStr">
+      <c r="E37" s="24" t="inlineStr">
         <is>
           <t>Evidence / location</t>
         </is>
       </c>
-      <c r="F37" s="23" t="inlineStr">
+      <c r="F37" s="24" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -1900,34 +2231,34 @@
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="22" t="inlineStr">
+      <c r="B44" s="23" t="inlineStr">
         <is>
           <t>Challenge tests</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="B45" s="23" t="inlineStr">
+      <c r="B45" s="24" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C45" s="23" t="inlineStr">
+      <c r="C45" s="24" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="D45" s="23" t="inlineStr">
+      <c r="D45" s="24" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="E45" s="23" t="inlineStr">
+      <c r="E45" s="24" t="inlineStr">
         <is>
           <t>Evidence / location</t>
         </is>
       </c>
-      <c r="F45" s="23" t="inlineStr">
+      <c r="F45" s="24" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -2019,34 +2350,34 @@
       </c>
     </row>
     <row r="52">
-      <c r="B52" s="22" t="inlineStr">
+      <c r="B52" s="23" t="inlineStr">
         <is>
           <t>Known failure modes</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="B53" s="23" t="inlineStr">
+      <c r="B53" s="24" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C53" s="23" t="inlineStr">
+      <c r="C53" s="24" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="D53" s="23" t="inlineStr">
+      <c r="D53" s="24" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="E53" s="23" t="inlineStr">
+      <c r="E53" s="24" t="inlineStr">
         <is>
           <t>Evidence / location</t>
         </is>
       </c>
-      <c r="F53" s="23" t="inlineStr">
+      <c r="F53" s="24" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -2138,34 +2469,34 @@
       </c>
     </row>
     <row r="60">
-      <c r="B60" s="22" t="inlineStr">
+      <c r="B60" s="23" t="inlineStr">
         <is>
           <t>Regulatory / methodological anchors</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="B61" s="23" t="inlineStr">
+      <c r="B61" s="24" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="C61" s="23" t="inlineStr">
+      <c r="C61" s="24" t="inlineStr">
         <is>
           <t>Scope</t>
         </is>
       </c>
-      <c r="D61" s="23" t="inlineStr">
+      <c r="D61" s="24" t="inlineStr">
         <is>
           <t>Source URL</t>
         </is>
       </c>
-      <c r="E61" s="23" t="inlineStr">
+      <c r="E61" s="24" t="inlineStr">
         <is>
           <t>Applicability</t>
         </is>
       </c>
-      <c r="F61" s="23" t="inlineStr">
+      <c r="F61" s="24" t="inlineStr">
         <is>
           <t>Review note</t>
         </is>
@@ -2279,49 +2610,49 @@
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" s="19" t="inlineStr">
+      <c r="B2" s="20" t="inlineStr">
         <is>
           <t>Independent Challenge, Override and Closure Log</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="23" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C4" s="23" t="inlineStr">
+      <c r="C4" s="24" t="inlineStr">
         <is>
           <t>Reviewer</t>
         </is>
       </c>
-      <c r="D4" s="23" t="inlineStr">
+      <c r="D4" s="24" t="inlineStr">
         <is>
           <t>Challenge</t>
         </is>
       </c>
-      <c r="E4" s="23" t="inlineStr">
+      <c r="E4" s="24" t="inlineStr">
         <is>
           <t>Owner response</t>
         </is>
       </c>
-      <c r="F4" s="23" t="inlineStr">
+      <c r="F4" s="24" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="G4" s="23" t="inlineStr">
+      <c r="G4" s="24" t="inlineStr">
         <is>
           <t>Impact</t>
         </is>
       </c>
-      <c r="H4" s="23" t="inlineStr">
+      <c r="H4" s="24" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I4" s="23" t="inlineStr">
+      <c r="I4" s="24" t="inlineStr">
         <is>
           <t>Closure</t>
         </is>
@@ -2454,54 +2785,54 @@
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" s="19" t="inlineStr">
+      <c r="B2" s="20" t="inlineStr">
         <is>
           <t>Source, Transformation, Ownership and Refresh Map</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="23" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>Source class</t>
         </is>
       </c>
-      <c r="C4" s="23" t="inlineStr">
+      <c r="C4" s="24" t="inlineStr">
         <is>
           <t>Cadence</t>
         </is>
       </c>
-      <c r="D4" s="23" t="inlineStr">
+      <c r="D4" s="24" t="inlineStr">
         <is>
           <t>Control</t>
         </is>
       </c>
-      <c r="E4" s="23" t="inlineStr">
+      <c r="E4" s="24" t="inlineStr">
         <is>
           <t>System / provider</t>
         </is>
       </c>
-      <c r="F4" s="23" t="inlineStr">
+      <c r="F4" s="24" t="inlineStr">
         <is>
           <t>As-of</t>
         </is>
       </c>
-      <c r="G4" s="23" t="inlineStr">
+      <c r="G4" s="24" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="H4" s="23" t="inlineStr">
+      <c r="H4" s="24" t="inlineStr">
         <is>
           <t>Transform</t>
         </is>
       </c>
-      <c r="I4" s="23" t="inlineStr">
+      <c r="I4" s="24" t="inlineStr">
         <is>
           <t>Downstream</t>
         </is>
       </c>
-      <c r="J4" s="23" t="inlineStr">
+      <c r="J4" s="24" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -2634,7 +2965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F19"/>
+  <dimension ref="B2:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3004,6 +3335,94 @@
         <v/>
       </c>
       <c r="F19" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Beginning remaining performance obligation (RPO)</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="n">
+        <v>950</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>950</v>
+      </c>
+      <c r="E20" s="10">
+        <f>IF(Cover!$C$9="Downside",D20,C20)</f>
+        <v/>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>$mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>RPO coverage of revenue (ending RPO / revenue)</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="D21" s="13" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E21" s="14">
+        <f>IF(Cover!$C$9="Downside",D21,C21)</f>
+        <v/>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Current portion of RPO (recognised within 12 months)</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="D22" s="11" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E22" s="12">
+        <f>IF(Cover!$C$9="Downside",D22,C22)</f>
+        <v/>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Contract liability / deferred revenue (% of revenue)</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D23" s="11" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E23" s="12">
+        <f>IF(Cover!$C$9="Downside",D23,C23)</f>
+        <v/>
+      </c>
+      <c r="F23" t="inlineStr">
         <is>
           <t>%</t>
         </is>
@@ -3210,28 +3629,28 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>Ending ARR</t>
         </is>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="16">
         <f>C5+C6+C7-C8-C9</f>
         <v/>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="16">
         <f>D5+D6+D7-D8-D9</f>
         <v/>
       </c>
-      <c r="E10" s="14">
+      <c r="E10" s="16">
         <f>E5+E6+E7-E8-E9</f>
         <v/>
       </c>
-      <c r="F10" s="14">
+      <c r="F10" s="16">
         <f>F5+F6+F7-F8-F9</f>
         <v/>
       </c>
-      <c r="G10" s="14">
+      <c r="G10" s="16">
         <f>G5+G6+G7-G8-G9</f>
         <v/>
       </c>
@@ -3464,28 +3883,28 @@
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>Total revenue</t>
         </is>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="16">
         <f>C5+C6</f>
         <v/>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" s="16">
         <f>D5+D6</f>
         <v/>
       </c>
-      <c r="E7" s="14">
+      <c r="E7" s="16">
         <f>E5+E6</f>
         <v/>
       </c>
-      <c r="F7" s="14">
+      <c r="F7" s="16">
         <f>F5+F6</f>
         <v/>
       </c>
-      <c r="G7" s="14">
+      <c r="G7" s="16">
         <f>G5+G6</f>
         <v/>
       </c>
@@ -3545,28 +3964,28 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>Total gross profit</t>
         </is>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="16">
         <f>C8+C9</f>
         <v/>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="16">
         <f>D8+D9</f>
         <v/>
       </c>
-      <c r="E10" s="14">
+      <c r="E10" s="16">
         <f>E8+E9</f>
         <v/>
       </c>
-      <c r="F10" s="14">
+      <c r="F10" s="16">
         <f>F8+F9</f>
         <v/>
       </c>
-      <c r="G10" s="14">
+      <c r="G10" s="16">
         <f>G8+G9</f>
         <v/>
       </c>
@@ -3680,28 +4099,28 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>Total operating expense</t>
         </is>
       </c>
-      <c r="C15" s="14">
+      <c r="C15" s="16">
         <f>C12+C13+C14</f>
         <v/>
       </c>
-      <c r="D15" s="14">
+      <c r="D15" s="16">
         <f>D12+D13+D14</f>
         <v/>
       </c>
-      <c r="E15" s="14">
+      <c r="E15" s="16">
         <f>E12+E13+E14</f>
         <v/>
       </c>
-      <c r="F15" s="14">
+      <c r="F15" s="16">
         <f>F12+F13+F14</f>
         <v/>
       </c>
-      <c r="G15" s="14">
+      <c r="G15" s="16">
         <f>G12+G13+G14</f>
         <v/>
       </c>
@@ -3896,28 +4315,28 @@
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="15" t="inlineStr">
         <is>
           <t>Free cash flow</t>
         </is>
       </c>
-      <c r="C23" s="14">
+      <c r="C23" s="16">
         <f>C16+C18-C21-C22</f>
         <v/>
       </c>
-      <c r="D23" s="14">
+      <c r="D23" s="16">
         <f>D16+D18-D21-D22</f>
         <v/>
       </c>
-      <c r="E23" s="14">
+      <c r="E23" s="16">
         <f>E16+E18-E21-E22</f>
         <v/>
       </c>
-      <c r="F23" s="14">
+      <c r="F23" s="16">
         <f>F16+F18-F21-F22</f>
         <v/>
       </c>
-      <c r="G23" s="14">
+      <c r="G23" s="16">
         <f>G16+G18-G21-G22</f>
         <v/>
       </c>
@@ -3963,7 +4382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H10"/>
+  <dimension ref="B2:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3978,14 +4397,14 @@
     <row r="2" ht="28" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Customer Acquisition Efficiency</t>
+          <t>Remaining Performance Obligations and Implied Bookings</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Metric</t>
+          <t>$mm</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
@@ -4017,162 +4436,352 @@
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>S&amp;M spend</t>
+          <t>Revenue recognised</t>
         </is>
       </c>
       <c r="C5" s="10">
-        <f>'Operating Model'!C12</f>
+        <f>'Operating Model'!C7</f>
         <v/>
       </c>
       <c r="D5" s="10">
-        <f>'Operating Model'!D12</f>
+        <f>'Operating Model'!D7</f>
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>'Operating Model'!E12</f>
+        <f>'Operating Model'!E7</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>'Operating Model'!F12</f>
+        <f>'Operating Model'!F7</f>
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>'Operating Model'!G12</f>
+        <f>'Operating Model'!G7</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>New + expansion ARR</t>
+          <t>Beginning RPO</t>
         </is>
       </c>
       <c r="C6" s="10">
-        <f>'ARR Rollforward'!C6+'ARR Rollforward'!C7</f>
+        <f>Assumptions!$E$20</f>
         <v/>
       </c>
       <c r="D6" s="10">
-        <f>'ARR Rollforward'!D6+'ARR Rollforward'!D7</f>
+        <f>C7</f>
         <v/>
       </c>
       <c r="E6" s="10">
-        <f>'ARR Rollforward'!E6+'ARR Rollforward'!E7</f>
+        <f>D7</f>
         <v/>
       </c>
       <c r="F6" s="10">
-        <f>'ARR Rollforward'!F6+'ARR Rollforward'!F7</f>
+        <f>E7</f>
         <v/>
       </c>
       <c r="G6" s="10">
-        <f>'ARR Rollforward'!G6+'ARR Rollforward'!G7</f>
+        <f>F7</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Magic number</t>
-        </is>
-      </c>
-      <c r="C7" s="15">
-        <f>IFERROR(C6/C5,0)</f>
-        <v/>
-      </c>
-      <c r="D7" s="15">
-        <f>IFERROR(D6/D5,0)</f>
-        <v/>
-      </c>
-      <c r="E7" s="15">
-        <f>IFERROR(E6/E5,0)</f>
-        <v/>
-      </c>
-      <c r="F7" s="15">
-        <f>IFERROR(F6/F5,0)</f>
-        <v/>
-      </c>
-      <c r="G7" s="15">
-        <f>IFERROR(G6/G5,0)</f>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Ending RPO</t>
+        </is>
+      </c>
+      <c r="C7" s="16">
+        <f>C5*Assumptions!$E$21</f>
+        <v/>
+      </c>
+      <c r="D7" s="16">
+        <f>D5*Assumptions!$E$21</f>
+        <v/>
+      </c>
+      <c r="E7" s="16">
+        <f>E5*Assumptions!$E$21</f>
+        <v/>
+      </c>
+      <c r="F7" s="16">
+        <f>F5*Assumptions!$E$21</f>
+        <v/>
+      </c>
+      <c r="G7" s="16">
+        <f>G5*Assumptions!$E$21</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAC payback (months)</t>
-        </is>
-      </c>
-      <c r="C8" s="16">
-        <f>IFERROR(C5/C6*12,0)</f>
-        <v/>
-      </c>
-      <c r="D8" s="16">
-        <f>IFERROR(D5/D6*12,0)</f>
-        <v/>
-      </c>
-      <c r="E8" s="16">
-        <f>IFERROR(E5/E6*12,0)</f>
-        <v/>
-      </c>
-      <c r="F8" s="16">
-        <f>IFERROR(F5/F6*12,0)</f>
-        <v/>
-      </c>
-      <c r="G8" s="16">
-        <f>IFERROR(G5/G6*12,0)</f>
+          <t>Implied gross bookings (residual)</t>
+        </is>
+      </c>
+      <c r="C8" s="10">
+        <f>C7-C6+C5</f>
+        <v/>
+      </c>
+      <c r="D8" s="10">
+        <f>D7-D6+D5</f>
+        <v/>
+      </c>
+      <c r="E8" s="10">
+        <f>E7-E6+E5</f>
+        <v/>
+      </c>
+      <c r="F8" s="10">
+        <f>F7-F6+F5</f>
+        <v/>
+      </c>
+      <c r="G8" s="10">
+        <f>G7-G6+G5</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>Gross-profit-weighted CAC payback (months)</t>
-        </is>
-      </c>
-      <c r="C9" s="16">
-        <f>IFERROR(C5/(C6*Assumptions!$E$19)*12,0)</f>
-        <v/>
-      </c>
-      <c r="D9" s="16">
-        <f>IFERROR(D5/(D6*Assumptions!$E$19)*12,0)</f>
-        <v/>
-      </c>
-      <c r="E9" s="16">
-        <f>IFERROR(E5/(E6*Assumptions!$E$19)*12,0)</f>
-        <v/>
-      </c>
-      <c r="F9" s="16">
-        <f>IFERROR(F5/(F6*Assumptions!$E$19)*12,0)</f>
-        <v/>
-      </c>
-      <c r="G9" s="16">
-        <f>IFERROR(G5/(G6*Assumptions!$E$19)*12,0)</f>
+          <t>Book-to-bill</t>
+        </is>
+      </c>
+      <c r="C9" s="14">
+        <f>IFERROR(C8/C5,0)</f>
+        <v/>
+      </c>
+      <c r="D9" s="14">
+        <f>IFERROR(D8/D5,0)</f>
+        <v/>
+      </c>
+      <c r="E9" s="14">
+        <f>IFERROR(E8/E5,0)</f>
+        <v/>
+      </c>
+      <c r="F9" s="14">
+        <f>IFERROR(F8/F5,0)</f>
+        <v/>
+      </c>
+      <c r="G9" s="14">
+        <f>IFERROR(G8/G5,0)</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>S&amp;M as % of new ARR</t>
+          <t>RPO growth</t>
         </is>
       </c>
       <c r="C10" s="12">
-        <f>IFERROR(C5/C6,0)</f>
+        <f>IFERROR(C7/C6-1,0)</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>IFERROR(D5/D6,0)</f>
+        <f>IFERROR(D7/D6-1,0)</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>IFERROR(E5/E6,0)</f>
+        <f>IFERROR(E7/E6-1,0)</f>
         <v/>
       </c>
       <c r="F10" s="12">
-        <f>IFERROR(F5/F6,0)</f>
+        <f>IFERROR(F7/F6-1,0)</f>
         <v/>
       </c>
       <c r="G10" s="12">
-        <f>IFERROR(G5/G6,0)</f>
+        <f>IFERROR(G7/G6-1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Current RPO (recognised within 12 months)</t>
+        </is>
+      </c>
+      <c r="C11" s="10">
+        <f>C7*Assumptions!$E$22</f>
+        <v/>
+      </c>
+      <c r="D11" s="10">
+        <f>D7*Assumptions!$E$22</f>
+        <v/>
+      </c>
+      <c r="E11" s="10">
+        <f>E7*Assumptions!$E$22</f>
+        <v/>
+      </c>
+      <c r="F11" s="10">
+        <f>F7*Assumptions!$E$22</f>
+        <v/>
+      </c>
+      <c r="G11" s="10">
+        <f>G7*Assumptions!$E$22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Non-current RPO</t>
+        </is>
+      </c>
+      <c r="C12" s="10">
+        <f>C7-C11</f>
+        <v/>
+      </c>
+      <c r="D12" s="10">
+        <f>D7-D11</f>
+        <v/>
+      </c>
+      <c r="E12" s="10">
+        <f>E7-E11</f>
+        <v/>
+      </c>
+      <c r="F12" s="10">
+        <f>F7-F11</f>
+        <v/>
+      </c>
+      <c r="G12" s="10">
+        <f>G7-G11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Contract liability (deferred revenue)</t>
+        </is>
+      </c>
+      <c r="C13" s="10">
+        <f>C5*Assumptions!$E$23</f>
+        <v/>
+      </c>
+      <c r="D13" s="10">
+        <f>D5*Assumptions!$E$23</f>
+        <v/>
+      </c>
+      <c r="E13" s="10">
+        <f>E5*Assumptions!$E$23</f>
+        <v/>
+      </c>
+      <c r="F13" s="10">
+        <f>F5*Assumptions!$E$23</f>
+        <v/>
+      </c>
+      <c r="G13" s="10">
+        <f>G5*Assumptions!$E$23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Unbilled RPO</t>
+        </is>
+      </c>
+      <c r="C14" s="10">
+        <f>C7-C13</f>
+        <v/>
+      </c>
+      <c r="D14" s="10">
+        <f>D7-D13</f>
+        <v/>
+      </c>
+      <c r="E14" s="10">
+        <f>E7-E13</f>
+        <v/>
+      </c>
+      <c r="F14" s="10">
+        <f>F7-F13</f>
+        <v/>
+      </c>
+      <c r="G14" s="10">
+        <f>G7-G13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Unbilled share of RPO</t>
+        </is>
+      </c>
+      <c r="C15" s="12">
+        <f>IFERROR(C14/C7,0)</f>
+        <v/>
+      </c>
+      <c r="D15" s="12">
+        <f>IFERROR(D14/D7,0)</f>
+        <v/>
+      </c>
+      <c r="E15" s="12">
+        <f>IFERROR(E14/E7,0)</f>
+        <v/>
+      </c>
+      <c r="F15" s="12">
+        <f>IFERROR(F14/F7,0)</f>
+        <v/>
+      </c>
+      <c r="G15" s="12">
+        <f>IFERROR(G14/G7,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Current RPO / following-year revenue</t>
+        </is>
+      </c>
+      <c r="C16" s="14">
+        <f>IFERROR(C11/'Operating Model'!D7,0)</f>
+        <v/>
+      </c>
+      <c r="D16" s="14">
+        <f>IFERROR(D11/'Operating Model'!E7,0)</f>
+        <v/>
+      </c>
+      <c r="E16" s="14">
+        <f>IFERROR(E11/'Operating Model'!F7,0)</f>
+        <v/>
+      </c>
+      <c r="F16" s="14">
+        <f>IFERROR(F11/'Operating Model'!G7,0)</f>
+        <v/>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Ending RPO / ending ARR</t>
+        </is>
+      </c>
+      <c r="C17" s="14">
+        <f>IFERROR(C7/'ARR Rollforward'!C10,0)</f>
+        <v/>
+      </c>
+      <c r="D17" s="14">
+        <f>IFERROR(D7/'ARR Rollforward'!D10,0)</f>
+        <v/>
+      </c>
+      <c r="E17" s="14">
+        <f>IFERROR(E7/'ARR Rollforward'!E10,0)</f>
+        <v/>
+      </c>
+      <c r="F17" s="14">
+        <f>IFERROR(F7/'ARR Rollforward'!F10,0)</f>
+        <v/>
+      </c>
+      <c r="G17" s="14">
+        <f>IFERROR(G7/'ARR Rollforward'!G10,0)</f>
         <v/>
       </c>
     </row>
@@ -4205,7 +4814,7 @@
     <row r="2" ht="28" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Growth versus Profitability Trade-off</t>
+          <t>Customer Acquisition Efficiency</t>
         </is>
       </c>
     </row>
@@ -4244,162 +4853,162 @@
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>Revenue growth</t>
-        </is>
-      </c>
-      <c r="C5" s="12">
-        <f>'ARR Rollforward'!C14</f>
-        <v/>
-      </c>
-      <c r="D5" s="12">
-        <f>IFERROR('Operating Model'!D7/'Operating Model'!C7-1,0)</f>
-        <v/>
-      </c>
-      <c r="E5" s="12">
-        <f>IFERROR('Operating Model'!E7/'Operating Model'!D7-1,0)</f>
-        <v/>
-      </c>
-      <c r="F5" s="12">
-        <f>IFERROR('Operating Model'!F7/'Operating Model'!E7-1,0)</f>
-        <v/>
-      </c>
-      <c r="G5" s="12">
-        <f>IFERROR('Operating Model'!G7/'Operating Model'!F7-1,0)</f>
+          <t>S&amp;M spend</t>
+        </is>
+      </c>
+      <c r="C5" s="10">
+        <f>'Operating Model'!C12</f>
+        <v/>
+      </c>
+      <c r="D5" s="10">
+        <f>'Operating Model'!D12</f>
+        <v/>
+      </c>
+      <c r="E5" s="10">
+        <f>'Operating Model'!E12</f>
+        <v/>
+      </c>
+      <c r="F5" s="10">
+        <f>'Operating Model'!F12</f>
+        <v/>
+      </c>
+      <c r="G5" s="10">
+        <f>'Operating Model'!G12</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>FCF margin</t>
-        </is>
-      </c>
-      <c r="C6" s="12">
-        <f>'Operating Model'!C24</f>
-        <v/>
-      </c>
-      <c r="D6" s="12">
-        <f>'Operating Model'!D24</f>
-        <v/>
-      </c>
-      <c r="E6" s="12">
-        <f>'Operating Model'!E24</f>
-        <v/>
-      </c>
-      <c r="F6" s="12">
-        <f>'Operating Model'!F24</f>
-        <v/>
-      </c>
-      <c r="G6" s="12">
-        <f>'Operating Model'!G24</f>
+          <t>New + expansion ARR</t>
+        </is>
+      </c>
+      <c r="C6" s="10">
+        <f>'ARR Rollforward'!C6+'ARR Rollforward'!C7</f>
+        <v/>
+      </c>
+      <c r="D6" s="10">
+        <f>'ARR Rollforward'!D6+'ARR Rollforward'!D7</f>
+        <v/>
+      </c>
+      <c r="E6" s="10">
+        <f>'ARR Rollforward'!E6+'ARR Rollforward'!E7</f>
+        <v/>
+      </c>
+      <c r="F6" s="10">
+        <f>'ARR Rollforward'!F6+'ARR Rollforward'!F7</f>
+        <v/>
+      </c>
+      <c r="G6" s="10">
+        <f>'ARR Rollforward'!G6+'ARR Rollforward'!G7</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>Rule of 40 (growth + FCF margin)</t>
-        </is>
-      </c>
-      <c r="C7" s="12">
-        <f>C5+C6</f>
-        <v/>
-      </c>
-      <c r="D7" s="12">
-        <f>D5+D6</f>
-        <v/>
-      </c>
-      <c r="E7" s="12">
-        <f>E5+E6</f>
-        <v/>
-      </c>
-      <c r="F7" s="12">
-        <f>F5+F6</f>
-        <v/>
-      </c>
-      <c r="G7" s="12">
-        <f>G5+G6</f>
+          <t>Magic number</t>
+        </is>
+      </c>
+      <c r="C7" s="14">
+        <f>IFERROR(C6/C5,0)</f>
+        <v/>
+      </c>
+      <c r="D7" s="14">
+        <f>IFERROR(D6/D5,0)</f>
+        <v/>
+      </c>
+      <c r="E7" s="14">
+        <f>IFERROR(E6/E5,0)</f>
+        <v/>
+      </c>
+      <c r="F7" s="14">
+        <f>IFERROR(F6/F5,0)</f>
+        <v/>
+      </c>
+      <c r="G7" s="14">
+        <f>IFERROR(G6/G5,0)</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>Non-GAAP operating margin</t>
-        </is>
-      </c>
-      <c r="C8" s="12">
-        <f>'Operating Model'!C20</f>
-        <v/>
-      </c>
-      <c r="D8" s="12">
-        <f>'Operating Model'!D20</f>
-        <v/>
-      </c>
-      <c r="E8" s="12">
-        <f>'Operating Model'!E20</f>
-        <v/>
-      </c>
-      <c r="F8" s="12">
-        <f>'Operating Model'!F20</f>
-        <v/>
-      </c>
-      <c r="G8" s="12">
-        <f>'Operating Model'!G20</f>
+          <t>CAC payback (months)</t>
+        </is>
+      </c>
+      <c r="C8" s="17">
+        <f>IFERROR(C5/C6*12,0)</f>
+        <v/>
+      </c>
+      <c r="D8" s="17">
+        <f>IFERROR(D5/D6*12,0)</f>
+        <v/>
+      </c>
+      <c r="E8" s="17">
+        <f>IFERROR(E5/E6*12,0)</f>
+        <v/>
+      </c>
+      <c r="F8" s="17">
+        <f>IFERROR(F5/F6*12,0)</f>
+        <v/>
+      </c>
+      <c r="G8" s="17">
+        <f>IFERROR(G5/G6*12,0)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rule of 40 (growth + operating margin)</t>
-        </is>
-      </c>
-      <c r="C9" s="12">
-        <f>C5+C8</f>
-        <v/>
-      </c>
-      <c r="D9" s="12">
-        <f>D5+D8</f>
-        <v/>
-      </c>
-      <c r="E9" s="12">
-        <f>E5+E8</f>
-        <v/>
-      </c>
-      <c r="F9" s="12">
-        <f>F5+F8</f>
-        <v/>
-      </c>
-      <c r="G9" s="12">
-        <f>G5+G8</f>
+          <t>Gross-profit-weighted CAC payback (months)</t>
+        </is>
+      </c>
+      <c r="C9" s="17">
+        <f>IFERROR(C5/(C6*Assumptions!$E$19)*12,0)</f>
+        <v/>
+      </c>
+      <c r="D9" s="17">
+        <f>IFERROR(D5/(D6*Assumptions!$E$19)*12,0)</f>
+        <v/>
+      </c>
+      <c r="E9" s="17">
+        <f>IFERROR(E5/(E6*Assumptions!$E$19)*12,0)</f>
+        <v/>
+      </c>
+      <c r="F9" s="17">
+        <f>IFERROR(F5/(F6*Assumptions!$E$19)*12,0)</f>
+        <v/>
+      </c>
+      <c r="G9" s="17">
+        <f>IFERROR(G5/(G6*Assumptions!$E$19)*12,0)</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C10">
-        <f>IF(C7&gt;=0.4,"PASS",IF(C7&gt;=0.3,"REVIEW","BELOW"))</f>
-        <v/>
-      </c>
-      <c r="D10">
-        <f>IF(D7&gt;=0.4,"PASS",IF(D7&gt;=0.3,"REVIEW","BELOW"))</f>
-        <v/>
-      </c>
-      <c r="E10">
-        <f>IF(E7&gt;=0.4,"PASS",IF(E7&gt;=0.3,"REVIEW","BELOW"))</f>
-        <v/>
-      </c>
-      <c r="F10">
-        <f>IF(F7&gt;=0.4,"PASS",IF(F7&gt;=0.3,"REVIEW","BELOW"))</f>
-        <v/>
-      </c>
-      <c r="G10">
-        <f>IF(G7&gt;=0.4,"PASS",IF(G7&gt;=0.3,"REVIEW","BELOW"))</f>
+          <t>S&amp;M as % of new ARR</t>
+        </is>
+      </c>
+      <c r="C10" s="12">
+        <f>IFERROR(C5/C6,0)</f>
+        <v/>
+      </c>
+      <c r="D10" s="12">
+        <f>IFERROR(D5/D6,0)</f>
+        <v/>
+      </c>
+      <c r="E10" s="12">
+        <f>IFERROR(E5/E6,0)</f>
+        <v/>
+      </c>
+      <c r="F10" s="12">
+        <f>IFERROR(F5/F6,0)</f>
+        <v/>
+      </c>
+      <c r="G10" s="12">
+        <f>IFERROR(G5/G6,0)</f>
         <v/>
       </c>
     </row>
@@ -4407,20 +5016,6 @@
   <mergeCells count="1">
     <mergeCell ref="B2:H2"/>
   </mergeCells>
-  <conditionalFormatting sqref="C10:G10">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>C10="PASS"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
-      <formula>C10="FAIL"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="3" dxfId="2">
-      <formula>C10="REVIEW"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="4" dxfId="1">
-      <formula>C10="BREACH"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>